<commit_message>
September checkpoint: rebalance v60/v70 targets (MOB down, ED/BD/Bride up), pull MOB launches back to 70/mo, add image-swap attribution and Jul-Sep cohort data
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/missacc_2027_growth_analysis/missacc_category_execution_map.xlsx
+++ b/missacc_2027_growth_analysis/missacc_category_execution_map.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>+50% / +60%</t>
+          <t>+50% / +55%(9月修订)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -556,8 +556,8 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>330 / 480款
-55或80/月全程平铺；12-3月不得停摆(今年该窗口仅68款是唯一执行事故)</t>
+          <t>330 / 420款
+55或70/月全程平铺;12-3月不得停摆(今年该窗口仅上68款是上半年唯一执行事故)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>【安全阀】动销率&lt;50%或单款收入连续两月恶化→回撤65-70/月，坑位还给BD</t>
+          <t>【安全阀·已启用】9月稀释黄灯(≤6月单产$909→$990→$674月化,7月实上95款超历史峰值62)→已回撤70/月;再恶化→60-65/月,坑位转Bride/ED</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>+80% / +95%</t>
+          <t>+80% / +100%(9月修订)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>【条件加码】10-11月达标→12-2月从ED挪5-10坑位/月；掉穿线→维持220不加</t>
+          <t>【条件加码】10-11月检查:动销率≥45%且单款≥$400→+100%维持且获MOB机动坑位10/月;未达→回落+95%。9月警示:同比+117%→+89%减速、客单价$109未向$90走、新款单产走低——检查前不加注</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>+65% / +80%</t>
+          <t>+65% / +86%(9月修订)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1,865个&gt;12月老款(动销率18.9%、单款$128)：长尾清理下架+腰部款换图换标题；动销率每+1pp≈+$9.5K/月</t>
+          <t>【已验证·第一优先】换图修复430款(5-9月,AI场景图为主):7月批次9月产出2.37x、8月批次1.78x vs 未换图控制组0.98x,净增~$3,160/天;老款池覆盖率仅10%(222/2300)→按批次扩量,单批换图后30天回报跌破成本即停;长尾清理下架继续</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>【触发条款】1月单款&lt;$450→目标下调至+45%/+55%，缺口转MOB/BM，2-3月坑位减15-20/月转BD</t>
+          <t>【双轨触发】1月双轨均未达(新款&lt;$450且存量轨衰减)→目标下调+45%/+55%;仅新款轨未达→回撤至+80%。10月复核换图批次回报是否衰减(台阶vs斜率)</t>
         </is>
       </c>
     </row>
@@ -690,12 +690,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>+35% / +42%</t>
+          <t>+35% / +43%(9月修订)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>池成熟+40%(Reviews复利)单独覆盖目标；爬坡≥6个月(第0月$241→第6月$515仍在涨)→今年的上新是2027H2/2028的收成；目标低于当前同比(+72%/+98%)</t>
+          <t>池成熟+40%(Reviews复利)单独覆盖目标；爬坡≥6个月(第0月$241→第6月$515仍在涨)→今年的上新是2027H2/2028的收成；目标低于当前同比(+72%/+98%);9月1-14同比+121%全盘唯一显著加速,目标沙袋最厚</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">

</xml_diff>